<commit_message>
updates downloads site, added bundles
</commit_message>
<xml_diff>
--- a/r2-uploads/sso-mapping-template.xlsx
+++ b/r2-uploads/sso-mapping-template.xlsx
@@ -1,41 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://omgww-my.sharepoint.com/personal/tamem_jalallar_ogilvy_com/Documents/Documents/TamemJ/TamemJ/r2-uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_FF530045FF7F714EA92C8F895BC30E3440025E08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30727602-B528-5245-AB6A-DB664CFF145A}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="11_FF530045FF7F714EA92C8F895BC30E3440025E08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17598069-8E40-734F-B6ED-9A8FE8BFB764}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15460" yWindow="-24320" windowWidth="36000" windowHeight="21420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>Okta / Entra SSO Mapping</t>
   </si>
   <si>
-    <t>Logo Placeholder</t>
-  </si>
-  <si>
-    <t>Organization Name IT Templates</t>
-  </si>
-  <si>
-    <t>Version 1.0 | Updated 2026-03-12 | Owner: IT Operations</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -112,13 +102,28 @@
   </si>
   <si>
     <t>Note Conditional Access requirements for access policy.</t>
+  </si>
+  <si>
+    <t>[LOGO]</t>
+  </si>
+  <si>
+    <t>Owner: IT Operations</t>
+  </si>
+  <si>
+    <t>[Organization Name] - IT Templates</t>
+  </si>
+  <si>
+    <t>Updated [DATE]</t>
+  </si>
+  <si>
+    <t>Version [1.0]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -249,6 +254,20 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="24"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -595,9 +614,23 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -643,7 +676,44 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -661,19 +731,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F80311A-C439-8A43-B5E9-32C5A4D695C7}" name="Table1" displayName="Table1" ref="A6:J18" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F80311A-C439-8A43-B5E9-32C5A4D695C7}" name="Table1" displayName="Table1" ref="A6:J18" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="A6:J18" xr:uid="{4F80311A-C439-8A43-B5E9-32C5A4D695C7}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{C0D6BEDA-4461-7044-A3E5-4BD9B1BE3608}" name="Application"/>
-    <tableColumn id="2" xr3:uid="{2DEF23D3-C71D-0D4E-B810-B3BF7055F16F}" name="Owner"/>
-    <tableColumn id="3" xr3:uid="{75EF73CA-5A6F-604B-9A54-DCBB473CAAB2}" name="SSO Protocol"/>
-    <tableColumn id="4" xr3:uid="{E4415D88-F87F-0A49-8D7C-417D4811F747}" name="SSO URL"/>
-    <tableColumn id="5" xr3:uid="{C7FC4709-A013-3749-9783-7800D5ABC4BE}" name="Entity ID"/>
-    <tableColumn id="6" xr3:uid="{973AECC8-AEC6-524F-B49D-E5E3CFB7F01F}" name="Claims Mapping"/>
-    <tableColumn id="7" xr3:uid="{918842C3-AE7D-944A-9EAB-0661B03BEE06}" name="Conditional Access"/>
-    <tableColumn id="8" xr3:uid="{ECBD59F0-A073-D24F-8F13-75EB8A2952F8}" name="Provisioning"/>
-    <tableColumn id="9" xr3:uid="{5C2C9D15-EA39-CA42-BFDF-AB39ADF42E8D}" name="Status"/>
-    <tableColumn id="10" xr3:uid="{77205B5B-73FB-0A4C-AC2E-88C2181ED94F}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{C0D6BEDA-4461-7044-A3E5-4BD9B1BE3608}" name="Application" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{2DEF23D3-C71D-0D4E-B810-B3BF7055F16F}" name="Owner" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{75EF73CA-5A6F-604B-9A54-DCBB473CAAB2}" name="SSO Protocol" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E4415D88-F87F-0A49-8D7C-417D4811F747}" name="SSO URL" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{C7FC4709-A013-3749-9783-7800D5ABC4BE}" name="Entity ID" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{973AECC8-AEC6-524F-B49D-E5E3CFB7F01F}" name="Claims Mapping" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{918842C3-AE7D-944A-9EAB-0661B03BEE06}" name="Conditional Access" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{ECBD59F0-A073-D24F-8F13-75EB8A2952F8}" name="Provisioning" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{5C2C9D15-EA39-CA42-BFDF-AB39ADF42E8D}" name="Status" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{77205B5B-73FB-0A4C-AC2E-88C2181ED94F}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -999,140 +1069,132 @@
   <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="10" width="24" customWidth="1"/>
+    <col min="1" max="2" width="24" style="3" customWidth="1"/>
+    <col min="3" max="3" width="10" style="3" customWidth="1"/>
+    <col min="4" max="4" width="31.5" style="3" customWidth="1"/>
+    <col min="5" max="10" width="24" style="3" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+    <row r="2" spans="1:10" ht="69" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
+    <row r="3" spans="1:10" ht="41" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
+      <c r="A4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>28</v>
+      </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="5" customFormat="1" ht="53" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="D6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="F6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D6" t="s">
+      <c r="G6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E6" t="s">
+      <c r="H6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F6" t="s">
+      <c r="I6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G6" t="s">
+      <c r="J6" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="H6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D7" t="s">
+      <c r="G7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E7" t="s">
+      <c r="H7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F7" t="s">
+      <c r="I7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="G7" t="s">
+      <c r="J7" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="H7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1151,32 +1213,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "updates downloads site, added bundles"
This reverts commit ab695179b7bce65e04b6ac121c2a0f1b7b88f706.
</commit_message>
<xml_diff>
--- a/r2-uploads/sso-mapping-template.xlsx
+++ b/r2-uploads/sso-mapping-template.xlsx
@@ -1,31 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://omgww-my.sharepoint.com/personal/tamem_jalallar_ogilvy_com/Documents/Documents/TamemJ/TamemJ/r2-uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="11_FF530045FF7F714EA92C8F895BC30E3440025E08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17598069-8E40-734F-B6ED-9A8FE8BFB764}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_FF530045FF7F714EA92C8F895BC30E3440025E08" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30727602-B528-5245-AB6A-DB664CFF145A}"/>
   <bookViews>
-    <workbookView xWindow="-15460" yWindow="-24320" windowWidth="36000" windowHeight="21420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Okta / Entra SSO Mapping</t>
   </si>
   <si>
+    <t>Logo Placeholder</t>
+  </si>
+  <si>
+    <t>Organization Name IT Templates</t>
+  </si>
+  <si>
+    <t>Version 1.0 | Updated 2026-03-12 | Owner: IT Operations</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -102,28 +112,13 @@
   </si>
   <si>
     <t>Note Conditional Access requirements for access policy.</t>
-  </si>
-  <si>
-    <t>[LOGO]</t>
-  </si>
-  <si>
-    <t>Owner: IT Operations</t>
-  </si>
-  <si>
-    <t>[Organization Name] - IT Templates</t>
-  </si>
-  <si>
-    <t>Updated [DATE]</t>
-  </si>
-  <si>
-    <t>Version [1.0]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -254,20 +249,6 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="24"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -614,23 +595,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -676,44 +643,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -731,19 +661,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F80311A-C439-8A43-B5E9-32C5A4D695C7}" name="Table1" displayName="Table1" ref="A6:J18" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F80311A-C439-8A43-B5E9-32C5A4D695C7}" name="Table1" displayName="Table1" ref="A6:J18" totalsRowShown="0">
   <autoFilter ref="A6:J18" xr:uid="{4F80311A-C439-8A43-B5E9-32C5A4D695C7}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{C0D6BEDA-4461-7044-A3E5-4BD9B1BE3608}" name="Application" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{2DEF23D3-C71D-0D4E-B810-B3BF7055F16F}" name="Owner" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{75EF73CA-5A6F-604B-9A54-DCBB473CAAB2}" name="SSO Protocol" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{E4415D88-F87F-0A49-8D7C-417D4811F747}" name="SSO URL" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{C7FC4709-A013-3749-9783-7800D5ABC4BE}" name="Entity ID" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{973AECC8-AEC6-524F-B49D-E5E3CFB7F01F}" name="Claims Mapping" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{918842C3-AE7D-944A-9EAB-0661B03BEE06}" name="Conditional Access" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{ECBD59F0-A073-D24F-8F13-75EB8A2952F8}" name="Provisioning" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{5C2C9D15-EA39-CA42-BFDF-AB39ADF42E8D}" name="Status" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{77205B5B-73FB-0A4C-AC2E-88C2181ED94F}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{C0D6BEDA-4461-7044-A3E5-4BD9B1BE3608}" name="Application"/>
+    <tableColumn id="2" xr3:uid="{2DEF23D3-C71D-0D4E-B810-B3BF7055F16F}" name="Owner"/>
+    <tableColumn id="3" xr3:uid="{75EF73CA-5A6F-604B-9A54-DCBB473CAAB2}" name="SSO Protocol"/>
+    <tableColumn id="4" xr3:uid="{E4415D88-F87F-0A49-8D7C-417D4811F747}" name="SSO URL"/>
+    <tableColumn id="5" xr3:uid="{C7FC4709-A013-3749-9783-7800D5ABC4BE}" name="Entity ID"/>
+    <tableColumn id="6" xr3:uid="{973AECC8-AEC6-524F-B49D-E5E3CFB7F01F}" name="Claims Mapping"/>
+    <tableColumn id="7" xr3:uid="{918842C3-AE7D-944A-9EAB-0661B03BEE06}" name="Conditional Access"/>
+    <tableColumn id="8" xr3:uid="{ECBD59F0-A073-D24F-8F13-75EB8A2952F8}" name="Provisioning"/>
+    <tableColumn id="9" xr3:uid="{5C2C9D15-EA39-CA42-BFDF-AB39ADF42E8D}" name="Status"/>
+    <tableColumn id="10" xr3:uid="{77205B5B-73FB-0A4C-AC2E-88C2181ED94F}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1069,132 +999,140 @@
   <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="24" style="3" customWidth="1"/>
-    <col min="3" max="3" width="10" style="3" customWidth="1"/>
-    <col min="4" max="4" width="31.5" style="3" customWidth="1"/>
-    <col min="5" max="10" width="24" style="3" customWidth="1"/>
-    <col min="11" max="16384" width="10.83203125" style="3"/>
+    <col min="1" max="10" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-    </row>
-    <row r="2" spans="1:10" ht="69" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="41" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
       <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="5" customFormat="1" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="5" t="s">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="E6" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="F6" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="G6" t="s">
         <v>11</v>
       </c>
+      <c r="H6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="A7" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="C7" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="D7" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="E7" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="F7" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="G7" t="s">
         <v>21</v>
       </c>
+      <c r="H7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" t="s">
+        <v>24</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A4:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1213,32 +1151,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>